<commit_message>
added 2025-26 even feedback faculty and subject details
</commit_message>
<xml_diff>
--- a/2025-Odd/2025 Odd.xlsx
+++ b/2025-Odd/2025 Odd.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/milav/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/milav/Code/StudentFeedbackAnalysis/2025-Odd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B2AF76E-6CBB-1B46-BD9A-17D1458537A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FC81F3-20FA-014C-8202-C0D342429C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{B17E0E1E-36A6-A148-BCCC-2BEDC95F523F}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" activeTab="1" xr2:uid="{B17E0E1E-36A6-A148-BCCC-2BEDC95F523F}"/>
   </bookViews>
   <sheets>
     <sheet name="master" sheetId="5" r:id="rId1"/>
+    <sheet name="sem1" sheetId="6" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1950" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2094" uniqueCount="140">
   <si>
     <t>Year</t>
   </si>
@@ -352,12 +353,117 @@
   <si>
     <t>24/11/2025</t>
   </si>
+  <si>
+    <t>KAP</t>
+  </si>
+  <si>
+    <t>DJM</t>
+  </si>
+  <si>
+    <t>MJV</t>
+  </si>
+  <si>
+    <t>FE</t>
+  </si>
+  <si>
+    <t>S&amp;Y</t>
+  </si>
+  <si>
+    <t>FEE</t>
+  </si>
+  <si>
+    <t>FICT</t>
+  </si>
+  <si>
+    <t>WDP</t>
+  </si>
+  <si>
+    <t>Mr. M J Vadhavaniya</t>
+  </si>
+  <si>
+    <t>Ms. K A Patel</t>
+  </si>
+  <si>
+    <t>Mr. D J Modi</t>
+  </si>
+  <si>
+    <t>24/07/2025</t>
+  </si>
+  <si>
+    <t>30/12/2025</t>
+  </si>
+  <si>
+    <t>DI01000051</t>
+  </si>
+  <si>
+    <t>Fundamentals of Electronics</t>
+  </si>
+  <si>
+    <t>DI01C00091</t>
+  </si>
+  <si>
+    <t>DI01000041</t>
+  </si>
+  <si>
+    <t>Sports and Yoga </t>
+  </si>
+  <si>
+    <t>DI01009011</t>
+  </si>
+  <si>
+    <t>Fundamentals of Electrical Engineering</t>
+  </si>
+  <si>
+    <t>DI01000091</t>
+  </si>
+  <si>
+    <t>DI01032011</t>
+  </si>
+  <si>
+    <t>Web Development Practice</t>
+  </si>
+  <si>
+    <t>Fundamentals of Information and Communication Technology</t>
+  </si>
+  <si>
+    <t>DI01000051: Fundamentals of Electronics By Dr. R N Patel</t>
+  </si>
+  <si>
+    <t>DI01C00091: Fundamentals of Information and Communication Technology By Mr. S P Joshiara</t>
+  </si>
+  <si>
+    <t>DI01000041: Sports and Yoga  By Mr. M J Vadhavaniya</t>
+  </si>
+  <si>
+    <t>DI01009011: Fundamentals of Electrical Engineering By Mr. N J Chauhan </t>
+  </si>
+  <si>
+    <t>DI01000091: Fundamentals of Information and Communication Technology By Mr. S J Chauhan</t>
+  </si>
+  <si>
+    <t>DI01000091: Fundamentals of Information and Communication Technology By Ms. M K Pedhadiya</t>
+  </si>
+  <si>
+    <t>DI01000091: Fundamentals of Information and Communication Technology By Mr. N J Chauhan </t>
+  </si>
+  <si>
+    <t>DI01032011: Web Development Practice By Mr. R C Parmar</t>
+  </si>
+  <si>
+    <t>DI01032011: Web Development Practice By Mr. M J Dabgar</t>
+  </si>
+  <si>
+    <t>DI01000041: Sports and Yoga  By Ms. K A Patel</t>
+  </si>
+  <si>
+    <t>DI01000041: Sports and Yoga  By Mr. D J Modi</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -369,6 +475,18 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -392,10 +510,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21258,4 +21378,582 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B60401D-BDC5-7542-9278-B7AE42BA8030}">
+  <dimension ref="A1:X24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="92.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="58.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F2" t="s">
+        <v>116</v>
+      </c>
+      <c r="G2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="K2" t="s">
+        <v>79</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G3" t="s">
+        <v>117</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" t="s">
+        <v>117</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="K4" t="s">
+        <v>107</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2025</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F5" t="s">
+        <v>116</v>
+      </c>
+      <c r="G5" t="s">
+        <v>117</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" t="s">
+        <v>116</v>
+      </c>
+      <c r="G6" t="s">
+        <v>117</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="K6" t="s">
+        <v>79</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2025</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="F7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G7" t="s">
+        <v>117</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K7" t="s">
+        <v>69</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2025</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G8" t="s">
+        <v>117</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G9" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K9" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2025</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F10" t="s">
+        <v>116</v>
+      </c>
+      <c r="G10" t="s">
+        <v>117</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="K10" t="s">
+        <v>28</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>2025</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F11" t="s">
+        <v>116</v>
+      </c>
+      <c r="G11" t="s">
+        <v>117</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="K11" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>2025</v>
+      </c>
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F12" t="s">
+        <v>116</v>
+      </c>
+      <c r="G12" t="s">
+        <v>117</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="K12" t="s">
+        <v>105</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>2025</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F13" t="s">
+        <v>116</v>
+      </c>
+      <c r="G13" t="s">
+        <v>117</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="K13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J24" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>